<commit_message>
Week 02 Day 04: Dynamic data analysis with UNIQUE SORT FILTER
</commit_message>
<xml_diff>
--- a/Month-01-Excel/Week-02/Day-03/Day-03-Data-Cleaning.xlsx
+++ b/Month-01-Excel/Week-02/Day-03/Day-03-Data-Cleaning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\4_MONTH\4-Month-Data-Analyst-Journey\Month-01-Excel\Week-02\Day-03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E49ACD5-7DC7-4735-B2BD-7C6893C784C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA4282F2-CAA9-4682-AA16-53EBAAA80167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="89">
   <si>
     <t>Customer_ID</t>
   </si>
@@ -320,6 +320,12 @@
   </si>
   <si>
     <t>Status: COMPLETED</t>
+  </si>
+  <si>
+    <t>Vhevk Csomet</t>
+  </si>
+  <si>
+    <t>vounyngnk</t>
   </si>
 </sst>
 </file>
@@ -400,7 +406,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -414,17 +420,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -990,7 +999,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C6CDE03-CE7F-4E18-897C-9D9D25213710}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="4" bestFit="1" customWidth="1"/>
@@ -1007,517 +1016,523 @@
     <col min="12" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="6" t="s">
         <v>42</v>
       </c>
       <c r="K1" s="8" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="L1" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="9">
         <v>22</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="4" t="b">
+      <c r="G2" s="9" t="b">
         <f>COUNTIF(B2:B13,B2)&gt;1</f>
         <v>1</v>
       </c>
-      <c r="H2" s="4" t="str">
+      <c r="H2" s="9" t="str">
         <f>IF(COUNTIF(B2:B13,B2)&gt;1,"Duplicate","Unique")</f>
         <v>Duplicate</v>
       </c>
-      <c r="I2" s="4" t="str">
+      <c r="I2" s="9" t="str">
         <f>IF(OR(LOWER(TRIM(F2))="active", LOWER(TRIM(F2))="act"), "Active", "Inactive")</f>
         <v>Active</v>
       </c>
-      <c r="J2" s="4" t="str" cm="1">
+      <c r="J2" s="9" t="str" cm="1">
         <f t="array" ref="J2">_xlfn.IFS(D2&lt;21,"Young",D2&lt;=25,"Adult",D2&gt;25,"Senior")</f>
         <v>Adult</v>
       </c>
-      <c r="K2" s="4" t="str">
+      <c r="K2" s="9" t="str">
         <f>IF(AND(TRIM(F2)="Active",D2&gt;=21),"Yes","No")</f>
         <v>Yes</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="L2" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="9">
         <v>24</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="4" t="b">
+      <c r="G3" s="9" t="b">
         <f t="shared" ref="G3:G13" si="0">COUNTIF(B3:B14,B3)&gt;1</f>
         <v>1</v>
       </c>
-      <c r="H3" s="4" t="str">
+      <c r="H3" s="9" t="str">
         <f t="shared" ref="H3:H13" si="1">IF(COUNTIF(B3:B14,B3)&gt;1,"Duplicate","Unique")</f>
         <v>Duplicate</v>
       </c>
-      <c r="I3" s="4" t="str">
+      <c r="I3" s="9" t="str">
         <f t="shared" ref="I3:I13" si="2">IF(OR(LOWER(TRIM(F3))="active", LOWER(TRIM(F3))="act"), "Active", "Inactive")</f>
         <v>Active</v>
       </c>
-      <c r="J3" s="4" t="str" cm="1">
+      <c r="J3" s="9" t="str" cm="1">
         <f t="array" ref="J3">_xlfn.IFS(D3&lt;21,"Young",D3&lt;=25,"Adult",D3&gt;25,"Senior")</f>
         <v>Adult</v>
       </c>
-      <c r="K3" s="4" t="str">
+      <c r="K3" s="9" t="str">
         <f t="shared" ref="K3:K13" si="3">IF(AND(TRIM(F3)="Active",D3&gt;=21),"Yes","No")</f>
         <v>Yes</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="9">
         <v>22</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="4" t="b">
+      <c r="G4" s="9" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H4" s="4" t="str">
+      <c r="H4" s="9" t="str">
         <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
-      <c r="I4" s="4" t="str">
+      <c r="I4" s="9" t="str">
         <f t="shared" si="2"/>
         <v>Active</v>
       </c>
-      <c r="J4" s="4" t="str" cm="1">
+      <c r="J4" s="9" t="str" cm="1">
         <f t="array" ref="J4">_xlfn.IFS(D4&lt;21,"Young",D4&lt;=25,"Adult",D4&gt;25,"Senior")</f>
         <v>Adult</v>
       </c>
-      <c r="K4" s="4" t="str">
+      <c r="K4" s="9" t="str">
         <f t="shared" si="3"/>
         <v>Yes</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="9">
         <v>19</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="4" t="b">
+      <c r="G5" s="9" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="9" t="str">
         <f t="shared" si="1"/>
         <v>Duplicate</v>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="9" t="str">
         <f t="shared" si="2"/>
         <v>Active</v>
       </c>
-      <c r="J5" s="4" t="str" cm="1">
+      <c r="J5" s="9" t="str" cm="1">
         <f t="array" ref="J5">_xlfn.IFS(D5&lt;21,"Young",D5&lt;=25,"Adult",D5&gt;25,"Senior")</f>
         <v>Young</v>
       </c>
-      <c r="K5" s="4" t="str">
+      <c r="K5" s="9" t="str">
         <f t="shared" si="3"/>
         <v>No</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="9">
         <v>21</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="4" t="b">
+      <c r="G6" s="9" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H6" s="4" t="str">
+      <c r="H6" s="9" t="str">
         <f t="shared" si="1"/>
         <v>Duplicate</v>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="9" t="str">
         <f t="shared" si="2"/>
         <v>Inactive</v>
       </c>
-      <c r="J6" s="4" t="str" cm="1">
+      <c r="J6" s="9" t="str" cm="1">
         <f t="array" ref="J6">_xlfn.IFS(D6&lt;21,"Young",D6&lt;=25,"Adult",D6&gt;25,"Senior")</f>
         <v>Adult</v>
       </c>
-      <c r="K6" s="4" t="str">
+      <c r="K6" s="9" t="str">
         <f t="shared" si="3"/>
         <v>No</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="9">
         <v>24</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="4" t="b">
+      <c r="G7" s="9" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H7" s="4" t="str">
+      <c r="H7" s="9" t="str">
         <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
-      <c r="I7" s="4" t="str">
+      <c r="I7" s="9" t="str">
         <f t="shared" si="2"/>
         <v>Active</v>
       </c>
-      <c r="J7" s="4" t="str" cm="1">
+      <c r="J7" s="9" t="str" cm="1">
         <f t="array" ref="J7">_xlfn.IFS(D7&lt;21,"Young",D7&lt;=25,"Adult",D7&gt;25,"Senior")</f>
         <v>Adult</v>
       </c>
-      <c r="K7" s="4" t="str">
+      <c r="K7" s="9" t="str">
         <f t="shared" si="3"/>
         <v>Yes</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="9">
         <v>25</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="4" t="b">
+      <c r="G8" s="9" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="4" t="str">
+      <c r="H8" s="9" t="str">
         <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
-      <c r="I8" s="4" t="str">
+      <c r="I8" s="9" t="str">
         <f t="shared" si="2"/>
         <v>Active</v>
       </c>
-      <c r="J8" s="4" t="str" cm="1">
+      <c r="J8" s="9" t="str" cm="1">
         <f t="array" ref="J8">_xlfn.IFS(D8&lt;21,"Young",D8&lt;=25,"Adult",D8&gt;25,"Senior")</f>
         <v>Adult</v>
       </c>
-      <c r="K8" s="4" t="str">
+      <c r="K8" s="9" t="str">
         <f t="shared" si="3"/>
         <v>Yes</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="9">
         <v>20</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="4" t="b">
+      <c r="G9" s="9" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H9" s="4" t="str">
+      <c r="H9" s="9" t="str">
         <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
-      <c r="I9" s="4" t="str">
+      <c r="I9" s="9" t="str">
         <f t="shared" si="2"/>
         <v>Active</v>
       </c>
-      <c r="J9" s="4" t="str" cm="1">
+      <c r="J9" s="9" t="str" cm="1">
         <f t="array" ref="J9">_xlfn.IFS(D9&lt;21,"Young",D9&lt;=25,"Adult",D9&gt;25,"Senior")</f>
         <v>Young</v>
       </c>
-      <c r="K9" s="4" t="str">
+      <c r="K9" s="9" t="str">
         <f t="shared" si="3"/>
         <v>No</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="9">
         <v>19</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="4" t="b">
+      <c r="G10" s="9" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="4" t="str">
+      <c r="H10" s="9" t="str">
         <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
-      <c r="I10" s="4" t="str">
+      <c r="I10" s="9" t="str">
         <f t="shared" si="2"/>
         <v>Active</v>
       </c>
-      <c r="J10" s="4" t="str" cm="1">
+      <c r="J10" s="9" t="str" cm="1">
         <f t="array" ref="J10">_xlfn.IFS(D10&lt;21,"Young",D10&lt;=25,"Adult",D10&gt;25,"Senior")</f>
         <v>Young</v>
       </c>
-      <c r="K10" s="4" t="str">
+      <c r="K10" s="9" t="str">
         <f t="shared" si="3"/>
         <v>No</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="9">
         <v>23</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G11" s="4" t="b">
+      <c r="G11" s="9" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H11" s="4" t="str">
+      <c r="H11" s="9" t="str">
         <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
-      <c r="I11" s="4" t="str">
+      <c r="I11" s="9" t="str">
         <f t="shared" si="2"/>
         <v>Active</v>
       </c>
-      <c r="J11" s="4" t="str" cm="1">
+      <c r="J11" s="9" t="str" cm="1">
         <f t="array" ref="J11">_xlfn.IFS(D11&lt;21,"Young",D11&lt;=25,"Adult",D11&gt;25,"Senior")</f>
         <v>Adult</v>
       </c>
-      <c r="K11" s="4" t="str">
+      <c r="K11" s="9" t="str">
         <f t="shared" si="3"/>
         <v>Yes</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="9">
         <v>27</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G12" s="4" t="b">
+      <c r="G12" s="9" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="4" t="str">
+      <c r="H12" s="9" t="str">
         <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
-      <c r="I12" s="4" t="str">
+      <c r="I12" s="9" t="str">
         <f t="shared" si="2"/>
         <v>Inactive</v>
       </c>
-      <c r="J12" s="4" t="str" cm="1">
+      <c r="J12" s="9" t="str" cm="1">
         <f t="array" ref="J12">_xlfn.IFS(D12&lt;21,"Young",D12&lt;=25,"Adult",D12&gt;25,"Senior")</f>
         <v>Senior</v>
       </c>
-      <c r="K12" s="4" t="str">
+      <c r="K12" s="9" t="str">
         <f t="shared" si="3"/>
         <v>No</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="9">
         <v>21</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="4" t="b">
+      <c r="G13" s="9" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H13" s="4" t="str">
+      <c r="H13" s="9" t="str">
         <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
-      <c r="I13" s="4" t="str">
+      <c r="I13" s="9" t="str">
         <f t="shared" si="2"/>
         <v>Inactive</v>
       </c>
-      <c r="J13" s="4" t="str" cm="1">
+      <c r="J13" s="9" t="str" cm="1">
         <f t="array" ref="J13">_xlfn.IFS(D13&lt;21,"Young",D13&lt;=25,"Adult",D13&gt;25,"Senior")</f>
         <v>Adult</v>
       </c>
-      <c r="K13" s="4" t="str">
+      <c r="K13" s="9" t="str">
         <f t="shared" si="3"/>
         <v>No</v>
       </c>
@@ -1550,16 +1565,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="7" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>